<commit_message>
version de test avec de vrai noms
</commit_message>
<xml_diff>
--- a/candidats.xlsx
+++ b/candidats.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -28,25 +28,16 @@
     <t xml:space="preserve">prenom</t>
   </si>
   <si>
-    <t xml:space="preserve">Naruto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uzumaki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">goku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">madara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uchiha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">roronoa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zoro</t>
+    <t xml:space="preserve">Tetang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ivan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabrielle</t>
   </si>
 </sst>
 </file>
@@ -61,6 +52,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -120,8 +112,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -252,41 +252,36 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>6</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>8</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Readme bien modifié, application fonctionnelle
</commit_message>
<xml_diff>
--- a/candidats.xlsx
+++ b/candidats.xlsx
@@ -112,16 +112,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -271,7 +267,7 @@
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Version avec les Statistiques en temps réelles.
</commit_message>
<xml_diff>
--- a/candidats.xlsx
+++ b/candidats.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -28,16 +28,25 @@
     <t xml:space="preserve">prenom</t>
   </si>
   <si>
+    <t xml:space="preserve">color</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tetang</t>
   </si>
   <si>
     <t xml:space="preserve">Ivan</t>
   </si>
   <si>
+    <t xml:space="preserve">blue</t>
+  </si>
+  <si>
     <t xml:space="preserve">Simo </t>
   </si>
   <si>
     <t xml:space="preserve">Gabrielle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">red</t>
   </si>
 </sst>
 </file>
@@ -112,12 +121,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -244,7 +257,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -254,21 +267,30 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>